<commit_message>
upgrade NSELECT==3 in CIGRE
</commit_message>
<xml_diff>
--- a/cable/cable_db.xlsx
+++ b/cable/cable_db.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26130"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\mario\python\pypacity\cable\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{239A288F-B9CD-4562-82A6-73600CA20A14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{257EE18E-E249-4CEE-BF59-99068BEFC324}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-24705" yWindow="1680" windowWidth="21600" windowHeight="11055" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-26925" yWindow="2055" windowWidth="28170" windowHeight="11055" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t>Cstring</t>
   </si>
@@ -76,6 +76,12 @@
   </si>
   <si>
     <t>10.4</t>
+  </si>
+  <si>
+    <t>TotalS</t>
+  </si>
+  <si>
+    <t>28.12</t>
   </si>
 </sst>
 </file>
@@ -393,13 +399,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N2"/>
+  <dimension ref="A1:O2"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.06640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="23.19921875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -442,13 +448,16 @@
       <c r="N1" t="s">
         <v>11</v>
       </c>
+      <c r="O1" t="s">
+        <v>17</v>
+      </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>12</v>
       </c>
-      <c r="B2">
-        <v>28.12</v>
+      <c r="B2" t="s">
+        <v>18</v>
       </c>
       <c r="C2" t="s">
         <v>16</v>
@@ -485,6 +494,9 @@
       </c>
       <c r="N2">
         <v>351.7</v>
+      </c>
+      <c r="O2">
+        <v>486.6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
# Fully functional version for IEEE 738 and CIGRE TB 601
</commit_message>
<xml_diff>
--- a/cable/cable_db.xlsx
+++ b/cable/cable_db.xlsx
@@ -1,31 +1,42 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26130"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26827"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\mario\python\pypacity\cable\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{257EE18E-E249-4CEE-BF59-99068BEFC324}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44E9B122-2DB3-473C-AFC8-594310EC0838}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-26925" yWindow="2055" windowWidth="28170" windowHeight="11055" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="1260" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="37">
   <si>
     <t>Cstring</t>
   </si>
@@ -72,16 +83,70 @@
     <t>4.44</t>
   </si>
   <si>
-    <t>C</t>
-  </si>
-  <si>
-    <t>10.4</t>
-  </si>
-  <si>
     <t>TotalS</t>
   </si>
   <si>
     <t>28.12</t>
+  </si>
+  <si>
+    <t>17.50</t>
+  </si>
+  <si>
+    <t>21.80</t>
+  </si>
+  <si>
+    <t>2.50</t>
+  </si>
+  <si>
+    <t>3.44</t>
+  </si>
+  <si>
+    <t>0.21993</t>
+  </si>
+  <si>
+    <t>0.07284</t>
+  </si>
+  <si>
+    <t>0.08689</t>
+  </si>
+  <si>
+    <t>0.5</t>
+  </si>
+  <si>
+    <t>1139.5</t>
+  </si>
+  <si>
+    <t>351.7</t>
+  </si>
+  <si>
+    <t>486.6</t>
+  </si>
+  <si>
+    <t>0.25197</t>
+  </si>
+  <si>
+    <t>0.13384</t>
+  </si>
+  <si>
+    <t>0.15707</t>
+  </si>
+  <si>
+    <t>379.81</t>
+  </si>
+  <si>
+    <t>128.16</t>
+  </si>
+  <si>
+    <t>623.22</t>
+  </si>
+  <si>
+    <t>147.22</t>
+  </si>
+  <si>
+    <t>LA-180</t>
+  </si>
+  <si>
+    <t>LA-280</t>
   </si>
 </sst>
 </file>
@@ -399,13 +464,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:N4"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.06640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="23.19921875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -413,90 +478,166 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" t="s">
+        <v>6</v>
+      </c>
+      <c r="I1" t="s">
+        <v>7</v>
+      </c>
+      <c r="J1" t="s">
+        <v>8</v>
+      </c>
+      <c r="K1" t="s">
+        <v>9</v>
+      </c>
+      <c r="L1" t="s">
+        <v>10</v>
+      </c>
+      <c r="M1" t="s">
+        <v>11</v>
+      </c>
+      <c r="N1" t="s">
         <v>15</v>
       </c>
-      <c r="D1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E1" t="s">
-        <v>2</v>
-      </c>
-      <c r="F1" t="s">
-        <v>3</v>
-      </c>
-      <c r="G1" t="s">
-        <v>4</v>
-      </c>
-      <c r="H1" t="s">
-        <v>5</v>
-      </c>
-      <c r="I1" t="s">
-        <v>6</v>
-      </c>
-      <c r="J1" t="s">
-        <v>7</v>
-      </c>
-      <c r="K1" t="s">
-        <v>8</v>
-      </c>
-      <c r="L1" t="s">
-        <v>9</v>
-      </c>
-      <c r="M1" t="s">
-        <v>10</v>
-      </c>
-      <c r="N1" t="s">
-        <v>11</v>
-      </c>
-      <c r="O1" t="s">
-        <v>17</v>
-      </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>12</v>
       </c>
       <c r="B2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D2">
+        <v>25</v>
+      </c>
+      <c r="E2">
+        <v>75</v>
+      </c>
+      <c r="F2">
+        <v>100</v>
+      </c>
+      <c r="G2" t="s">
+        <v>22</v>
+      </c>
+      <c r="H2" t="s">
+        <v>23</v>
+      </c>
+      <c r="I2" t="s">
+        <v>24</v>
+      </c>
+      <c r="J2" t="s">
+        <v>24</v>
+      </c>
+      <c r="K2">
+        <v>3</v>
+      </c>
+      <c r="L2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M2" t="s">
+        <v>26</v>
+      </c>
+      <c r="N2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="A3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D3">
+        <v>5</v>
+      </c>
+      <c r="E3">
+        <v>85</v>
+      </c>
+      <c r="F3">
+        <v>100</v>
+      </c>
+      <c r="G3" t="s">
+        <v>21</v>
+      </c>
+      <c r="H3" t="s">
+        <v>28</v>
+      </c>
+      <c r="I3" t="s">
+        <v>24</v>
+      </c>
+      <c r="J3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K3">
+        <v>2</v>
+      </c>
+      <c r="L3" t="s">
+        <v>31</v>
+      </c>
+      <c r="M3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="A4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B4" t="s">
         <v>18</v>
       </c>
-      <c r="C2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E2">
-        <v>25</v>
-      </c>
-      <c r="F2">
-        <v>75</v>
-      </c>
-      <c r="G2">
+      <c r="C4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D4">
+        <v>5</v>
+      </c>
+      <c r="E4">
+        <v>85</v>
+      </c>
+      <c r="F4">
         <v>100</v>
       </c>
-      <c r="H2">
-        <v>7.2840000000000002E-2</v>
-      </c>
-      <c r="I2">
-        <v>8.6889999999999995E-2</v>
-      </c>
-      <c r="J2">
-        <v>0.5</v>
-      </c>
-      <c r="K2">
-        <v>0.5</v>
-      </c>
-      <c r="L2">
-        <v>3</v>
-      </c>
-      <c r="M2">
-        <v>1139.5</v>
-      </c>
-      <c r="N2">
-        <v>351.7</v>
-      </c>
-      <c r="O2">
-        <v>486.6</v>
+      <c r="G4" t="s">
+        <v>29</v>
+      </c>
+      <c r="H4" t="s">
+        <v>30</v>
+      </c>
+      <c r="I4" t="s">
+        <v>24</v>
+      </c>
+      <c r="J4" t="s">
+        <v>24</v>
+      </c>
+      <c r="K4">
+        <v>2</v>
+      </c>
+      <c r="L4" t="s">
+        <v>33</v>
+      </c>
+      <c r="M4" t="s">
+        <v>34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>